<commit_message>
Modelo de consumo validado wuju
</commit_message>
<xml_diff>
--- a/data/validacion/elmo_data.xlsx
+++ b/data/validacion/elmo_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECNO-MASTER\Desktop\Elmo_infrastructure_sizing_NP-\data\validacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E43B2F08-B73A-4E6D-B37B-A88C928931F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACE06941-5D23-41C7-B655-A886FB6760C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1860" yWindow="1860" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1860" yWindow="1860" windowWidth="21600" windowHeight="11295" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Batteries" sheetId="1" r:id="rId1"/>
@@ -3952,7 +3952,7 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>1750</v>
+        <v>10000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
carga ob validada con WP1
</commit_message>
<xml_diff>
--- a/data/validacion/elmo_data.xlsx
+++ b/data/validacion/elmo_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECNO-MASTER\Desktop\Elmo_infrastructure_sizing_NP-\data\validacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64893990-1730-44E6-A831-42B9408AE7E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D6AF9DE-CB62-4B48-B118-C3702A8BA4CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1860" yWindow="1860" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3946,13 +3946,13 @@
         <v>0</v>
       </c>
       <c r="E3">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F3">
         <v>0</v>
       </c>
       <c r="G3">
-        <v>4000</v>
+        <v>5000</v>
       </c>
     </row>
   </sheetData>
@@ -4023,7 +4023,7 @@
         <v>1</v>
       </c>
       <c r="F3">
-        <v>4000</v>
+        <v>5000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
condiciones de borde y rest max swaps son compatibles, falta cerrar gap 15%, y meter solucion del fijo en variable
</commit_message>
<xml_diff>
--- a/data/validacion/elmo_data.xlsx
+++ b/data/validacion/elmo_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECNO-MASTER\Desktop\Elmo_infrastructure_sizing_NP-\data\validacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88CB3438-6C30-4D43-80C0-A226E46D2F27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D96B753B-53FA-4DEE-88B8-CEFF302DB259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1860" yWindow="1860" windowWidth="21600" windowHeight="11295" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Batteries" sheetId="1" r:id="rId1"/>
@@ -4151,7 +4151,7 @@
         <v>1</v>
       </c>
       <c r="F3">
-        <v>2100</v>
+        <v>5000</v>
       </c>
       <c r="G3">
         <v>5000</v>

</xml_diff>